<commit_message>
Add: Testes 1 - 3 da automação
</commit_message>
<xml_diff>
--- a/cadastrar.xlsx
+++ b/cadastrar.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
   <si>
     <t>ID Processo</t>
   </si>
@@ -35,71 +35,38 @@
     <t>Base Código</t>
   </si>
   <si>
-    <t>883858</t>
-  </si>
-  <si>
-    <t>23.278.436-1</t>
-  </si>
-  <si>
-    <t>VCP</t>
-  </si>
-  <si>
-    <t>PMW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23.214.581-4 </t>
-  </si>
-  <si>
     <t>CGH</t>
   </si>
   <si>
-    <t>23.332.641-3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sede Azul </t>
-  </si>
-  <si>
-    <t>968357</t>
-  </si>
-  <si>
-    <t>23.330.612-9</t>
-  </si>
-  <si>
-    <t>23.339.175-4</t>
-  </si>
-  <si>
-    <t>JTC</t>
-  </si>
-  <si>
-    <t>23.339.176-2</t>
-  </si>
-  <si>
-    <t>ARU</t>
-  </si>
-  <si>
-    <t>23.339.177-1</t>
-  </si>
-  <si>
-    <t>MII</t>
-  </si>
-  <si>
-    <t>23.339.178-9</t>
-  </si>
-  <si>
-    <t>RAO</t>
-  </si>
-  <si>
-    <t>23.339.179-7</t>
-  </si>
-  <si>
-    <t>SJP</t>
+    <t>R3THJPP367HJR9</t>
+  </si>
+  <si>
+    <t>MOC</t>
+  </si>
+  <si>
+    <t>RKFHJ2S3XISF4N</t>
+  </si>
+  <si>
+    <t>RL4HIY6FPJYA8T</t>
+  </si>
+  <si>
+    <t>RF3HK5IXCW56QA</t>
+  </si>
+  <si>
+    <t>THE</t>
+  </si>
+  <si>
+    <t>Processo</t>
+  </si>
+  <si>
+    <t>FISCALIZAÇÃO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -110,6 +77,13 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -129,7 +103,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -152,22 +126,34 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFFFD966"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFFFD966"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFFD966"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFD966"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -450,15 +436,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="34.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -468,105 +455,77 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>3</v>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="3">
+        <v>984857</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>5</v>
       </c>
+      <c r="D2" s="3" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
-        <v>901558</v>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>984859</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
+        <v>984869</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>6</v>
+      <c r="C4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
-        <v>967759</v>
-      </c>
-      <c r="B4" s="3" t="s">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
+        <v>984871</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>8</v>
+      <c r="D5" s="3" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>10</v>
-      </c>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="3"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="4">
-        <v>973410</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="4">
-        <v>973412</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="4">
-        <v>973413</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="4">
-        <v>973415</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="4">
-        <v>973417</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>22</v>
-      </c>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -775,15 +734,15 @@
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5CBD717-E7CA-471D-A675-1E703ACDF3D5}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="cdc37f11-6699-4390-935e-7d00f6a9cb17"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Alterações gerais e organização
</commit_message>
<xml_diff>
--- a/cadastrar.xlsx
+++ b/cadastrar.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
   <si>
     <t>ID Processo</t>
   </si>
@@ -38,28 +38,31 @@
     <t>CGH</t>
   </si>
   <si>
-    <t>R3THJPP367HJR9</t>
-  </si>
-  <si>
-    <t>MOC</t>
-  </si>
-  <si>
-    <t>RKFHJ2S3XISF4N</t>
-  </si>
-  <si>
     <t>RL4HIY6FPJYA8T</t>
   </si>
   <si>
-    <t>RF3HK5IXCW56QA</t>
-  </si>
-  <si>
-    <t>THE</t>
-  </si>
-  <si>
     <t>Processo</t>
   </si>
   <si>
     <t>FISCALIZAÇÃO</t>
+  </si>
+  <si>
+    <t>RL4HIY6E48Y5TW</t>
+  </si>
+  <si>
+    <t>RH0HJJERDQECU9</t>
+  </si>
+  <si>
+    <t>Call Center - Belo Horizonte</t>
+  </si>
+  <si>
+    <t>S1VHJJ8FYNHI73</t>
+  </si>
+  <si>
+    <t>PVH</t>
+  </si>
+  <si>
+    <t>Sede Azul</t>
   </si>
 </sst>
 </file>
@@ -145,12 +148,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -436,7 +436,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -456,76 +456,64 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="3">
-        <v>984857</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>11</v>
+      <c r="A2" s="2">
+        <v>937555</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="3">
-        <v>984859</v>
-      </c>
-      <c r="B3" s="3" t="s">
+      <c r="A3" s="2">
+        <v>937655</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>6</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
-        <v>984869</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>11</v>
+      <c r="A4" s="2">
+        <v>959555</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="3">
-        <v>984871</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="3" t="s">
+      <c r="A5" s="2">
+        <v>959559</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="3"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="3"/>
+      <c r="D5" s="2" t="s">
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -533,23 +521,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="cdc37f11-6699-4390-935e-7d00f6a9cb17" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010040810410046D4846AFC1D9D1724EAE0C" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3cf92e38dbd5ca6e29a3dbc90f9259c3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="cdc37f11-6699-4390-935e-7d00f6a9cb17" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3b7840fd93bba6919c464d2db268669e" ns3:_="">
     <xsd:import namespace="cdc37f11-6699-4390-935e-7d00f6a9cb17"/>
@@ -731,31 +702,24 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="cdc37f11-6699-4390-935e-7d00f6a9cb17" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5CBD717-E7CA-471D-A675-1E703ACDF3D5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="cdc37f11-6699-4390-935e-7d00f6a9cb17"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D2E150F-7C48-466A-AA6B-C8C58D0A952D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9964EC62-F762-492F-9669-9C56E6C51FCE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -771,4 +735,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D2E150F-7C48-466A-AA6B-C8C58D0A952D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5CBD717-E7CA-471D-A675-1E703ACDF3D5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="cdc37f11-6699-4390-935e-7d00f6a9cb17"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>